<commit_message>
updated importer to handle units
also fixed a small issue with regexing formulas in SDS.
</commit_message>
<xml_diff>
--- a/test_import.xlsx
+++ b/test_import.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{099EFCF0-47D8-4668-849F-1B819E3E63DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{15659987-BF7F-4B99-A59F-8F34B386D675}"/>
+    <workbookView minimized="1" xWindow="1044" yWindow="1044" windowWidth="2388" windowHeight="564" xr2:uid="{15659987-BF7F-4B99-A59F-8F34B386D675}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$H$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Sheet1!$1:$1</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -239,7 +239,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -253,17 +253,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -586,11 +580,11 @@
   <cols>
     <col min="1" max="1" width="33.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="16" style="4" customWidth="1"/>
-    <col min="3" max="3" width="11.44140625" style="10" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" style="8" customWidth="1"/>
     <col min="4" max="4" width="11" style="1" customWidth="1"/>
     <col min="5" max="5" width="12.109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="9.109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9.33203125" style="5" customWidth="1"/>
+    <col min="7" max="7" width="9.33203125" style="4" customWidth="1"/>
     <col min="8" max="8" width="10.88671875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -601,7 +595,7 @@
       <c r="B1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="7" t="s">
         <v>23</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -613,10 +607,10 @@
       <c r="F1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -627,7 +621,7 @@
       <c r="B2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="8" t="s">
         <v>25</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -639,7 +633,7 @@
       <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="4" t="s">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -653,7 +647,7 @@
       <c r="B3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -668,7 +662,7 @@
       <c r="G3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H3" s="5">
         <v>41435</v>
       </c>
     </row>
@@ -679,7 +673,7 @@
       <c r="B4" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="9" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -691,10 +685,10 @@
       <c r="F4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="5">
         <v>42376</v>
       </c>
     </row>
@@ -705,7 +699,7 @@
       <c r="B5" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="8" t="s">
         <v>26</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -731,7 +725,7 @@
       <c r="B6" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="8" t="s">
         <v>31</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -746,7 +740,7 @@
       <c r="G6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="5">
         <v>43850</v>
       </c>
     </row>
@@ -757,7 +751,7 @@
       <c r="B7" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -772,7 +766,7 @@
       <c r="G7" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="5">
         <v>42171</v>
       </c>
     </row>
@@ -783,7 +777,7 @@
       <c r="B8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="8" t="s">
         <v>27</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -798,7 +792,7 @@
       <c r="G8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="5">
         <v>44071</v>
       </c>
     </row>

</xml_diff>